<commit_message>
deploy: main → b4f471f267fdeb9a01e1bc613f07326d28311907
</commit_message>
<xml_diff>
--- a/StructureDefinition-IneraIndexEntry.xlsx
+++ b/StructureDefinition-IneraIndexEntry.xlsx
@@ -490,7 +490,7 @@
 </t>
   </si>
   <si>
-    <t>Security Labels applied to this resource</t>
+    <t>Säkerhetsetiketter som FHIR-EI tillämpar per syfte, t.ex. NOPAT</t>
   </si>
   <si>
     <t>Security labels applied to this resource. These tags connect specific resources to the overall security policy and infrastructure.</t>
@@ -4290,7 +4290,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="11" hidden="true">
+    <row r="11">
       <c r="A11" t="s" s="2">
         <v>149</v>
       </c>
@@ -4309,7 +4309,7 @@
         <v>83</v>
       </c>
       <c r="H11" t="s" s="2">
-        <v>81</v>
+        <v>97</v>
       </c>
       <c r="I11" t="s" s="2">
         <v>81</v>

</xml_diff>